<commit_message>
fix errors in verify-2025 and baseline TEW scenarios
</commit_message>
<xml_diff>
--- a/data/data_analysis/understanding TEW markets.xlsx
+++ b/data/data_analysis/understanding TEW markets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\data\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADFBF5DD-921A-48E9-AD3B-796B8FDF0B4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7601D9F5-C6EC-4AEA-AFA7-70CD0754EB8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{8111BAC2-3C26-4A41-BBD5-6F57C9F53EF0}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="124">
   <si>
     <t>2025 dollars</t>
   </si>
@@ -318,9 +318,6 @@
     <t>2025$/t CDR</t>
   </si>
   <si>
-    <t>Fixed solution</t>
-  </si>
-  <si>
     <t>Cost Breakdown</t>
   </si>
   <si>
@@ -406,6 +403,15 @@
   </si>
   <si>
     <t>Updated CDR yield</t>
+  </si>
+  <si>
+    <t>$/ton-km</t>
+  </si>
+  <si>
+    <t>Test 2 - issue was that I didn't update coefficients in scenarios without transportation cost reduction</t>
+  </si>
+  <si>
+    <t>Updated Version</t>
   </si>
 </sst>
 </file>
@@ -1133,6 +1139,309 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$L$62</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2025 dollars</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-1EAF-4FDA-A9E0-5EB18149C531}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-1EAF-4FDA-A9E0-5EB18149C531}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-1EAF-4FDA-A9E0-5EB18149C531}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-1EAF-4FDA-A9E0-5EB18149C531}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-1EAF-4FDA-A9E0-5EB18149C531}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$K$63:$K$67</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Silicate</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Electricity</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Cropland</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Freight</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Non-Input</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$L$63:$L$67</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>8.9466666666666653E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.4554365567999997E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.6839999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.8826871597348834E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.26839999999999997</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000A-1EAF-4FDA-A9E0-5EB18149C531}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1213,6 +1522,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
   <cs:axisTitle>
@@ -1733,6 +2082,525 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2413,6 +3281,83 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>118</xdr:row>
+      <xdr:rowOff>33337</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>132</xdr:row>
+      <xdr:rowOff>109537</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{743113F5-47E6-4352-B68D-06B42B1A496E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>115</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4638675" cy="1561636"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3CFFB3AC-384E-431A-BD37-5B897A120972}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="12573000"/>
+          <a:ext cx="4638675" cy="1561636"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2733,7 +3678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E8CADC1-B46D-415F-8453-53E8EF7749F4}">
-  <dimension ref="A1:N84"/>
+  <dimension ref="A1:N133"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.140625" bestFit="1" customWidth="1"/>
@@ -2752,7 +3697,7 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -3154,7 +4099,7 @@
         <v>5.8666669999999999E-3</v>
       </c>
       <c r="C17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>18</v>
@@ -3331,7 +4276,7 @@
         <v>66</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L24" s="5" t="s">
         <v>0</v>
@@ -3372,7 +4317,7 @@
         <v>2.255040360065466E-3</v>
       </c>
       <c r="K25" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L25">
         <f>C6*G18</f>
@@ -3410,7 +4355,7 @@
         <v>2.6642056628477899E-3</v>
       </c>
       <c r="K26" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L26">
         <f>C22*G18</f>
@@ -3434,7 +4379,7 @@
         <v>-2.2562876799999999E-3</v>
       </c>
       <c r="K27" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L27">
         <f>H11*G19</f>
@@ -3443,7 +4388,7 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="K28" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L28">
         <f>H14*G20*G21</f>
@@ -3455,7 +4400,7 @@
         <v>69</v>
       </c>
       <c r="K29" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L29">
         <f>M12</f>
@@ -3574,7 +4519,7 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -4006,7 +4951,7 @@
         <v>72</v>
       </c>
       <c r="K57" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
@@ -4099,10 +5044,10 @@
         <v>75</v>
       </c>
       <c r="F60" t="s">
+        <v>98</v>
+      </c>
+      <c r="G60" t="s">
         <v>99</v>
-      </c>
-      <c r="G60" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
@@ -4126,7 +5071,7 @@
         <v>62</v>
       </c>
       <c r="K62" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L62" s="5" t="s">
         <v>0</v>
@@ -4150,7 +5095,7 @@
         <v>66</v>
       </c>
       <c r="K63" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L63">
         <f>C44*G56</f>
@@ -4174,7 +5119,7 @@
         <v>1.272150909090909E-3</v>
       </c>
       <c r="K64" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L64">
         <f>C60*G56</f>
@@ -4198,7 +5143,7 @@
         <v>0.41636306000000006</v>
       </c>
       <c r="K65" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L65">
         <f>H49*G57</f>
@@ -4222,7 +5167,7 @@
         <v>-2.2562876799999999E-3</v>
       </c>
       <c r="K66" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L66">
         <f>H52*G58*G59</f>
@@ -4231,7 +5176,7 @@
     </row>
     <row r="67" spans="6:12" x14ac:dyDescent="0.25">
       <c r="K67" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L67">
         <f>M50</f>
@@ -4323,122 +5268,122 @@
     </row>
     <row r="75" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F75" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="76" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F76" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G76" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="G76" s="5" t="s">
-        <v>105</v>
       </c>
       <c r="H76" s="5" t="s">
         <v>2</v>
       </c>
       <c r="I76" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="77" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F77" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G77">
         <f>G18/G19</f>
         <v>0.5</v>
       </c>
       <c r="H77" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I77" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="78" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F78" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G78">
         <v>40</v>
       </c>
       <c r="H78" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I78" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="79" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F79" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G79">
         <f>G18</f>
         <v>12.22</v>
       </c>
       <c r="H79" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I79" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="80" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F80" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G80">
         <f>4*44/12</f>
         <v>14.666666666666666</v>
       </c>
       <c r="H80" t="s">
+        <v>111</v>
+      </c>
+      <c r="I80" t="s">
+        <v>108</v>
+      </c>
+      <c r="J80" t="s">
         <v>112</v>
       </c>
-      <c r="I80" t="s">
-        <v>109</v>
-      </c>
-      <c r="J80" t="s">
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F81" t="s">
         <v>113</v>
-      </c>
-    </row>
-    <row r="81" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F81" t="s">
-        <v>114</v>
       </c>
       <c r="G81">
         <v>18</v>
       </c>
       <c r="H81" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="82" spans="6:8" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F82" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G82">
         <v>1.6</v>
       </c>
       <c r="H82" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="83" spans="6:8" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F83" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G83">
         <f>(G81+G82)*0.0036/1000</f>
         <v>7.0560000000000002E-5</v>
       </c>
       <c r="H83" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="84" spans="6:8" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F84" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G84">
         <f>B17</f>
@@ -4449,9 +5394,886 @@
         <v>EJ/Mt crushed silicate</v>
       </c>
     </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A88" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A89" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K89" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A90" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B90" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C90" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F90" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G90" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H90" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K90" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L90" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M90" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>53</v>
+      </c>
+      <c r="B91">
+        <v>69.248999999999995</v>
+      </c>
+      <c r="C91" t="s">
+        <v>41</v>
+      </c>
+      <c r="F91" t="s">
+        <v>16</v>
+      </c>
+      <c r="G91">
+        <v>0.193</v>
+      </c>
+      <c r="H91" t="s">
+        <v>41</v>
+      </c>
+      <c r="K91" t="s">
+        <v>24</v>
+      </c>
+      <c r="L91">
+        <v>0.17699999999999999</v>
+      </c>
+      <c r="M91" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A92" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B92" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C92" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D92" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E92" s="5"/>
+      <c r="F92" t="s">
+        <v>17</v>
+      </c>
+      <c r="G92">
+        <v>8.1720000000000006</v>
+      </c>
+      <c r="H92" t="s">
+        <v>23</v>
+      </c>
+      <c r="K92" t="s">
+        <v>26</v>
+      </c>
+      <c r="L92">
+        <v>4.2290000000000001E-2</v>
+      </c>
+      <c r="M92" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>54</v>
+      </c>
+      <c r="B93">
+        <v>1E-3</v>
+      </c>
+      <c r="C93">
+        <f>B93*6.1</f>
+        <v>6.0999999999999995E-3</v>
+      </c>
+      <c r="D93" t="s">
+        <v>56</v>
+      </c>
+      <c r="F93" t="s">
+        <v>52</v>
+      </c>
+      <c r="G93">
+        <v>0.38700000000000001</v>
+      </c>
+      <c r="H93" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K94" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L94" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="M94" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="N94" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A95" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F95" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G95" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="H95" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="I95" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="K95" t="s">
+        <v>1</v>
+      </c>
+      <c r="L95">
+        <v>1.147</v>
+      </c>
+      <c r="M95">
+        <f>L95*6.1</f>
+        <v>6.9966999999999997</v>
+      </c>
+      <c r="N95" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A96" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C96" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F96" t="s">
+        <v>4</v>
+      </c>
+      <c r="G96">
+        <v>0.66900000000000004</v>
+      </c>
+      <c r="H96">
+        <f>G96*6.1</f>
+        <v>4.0808999999999997</v>
+      </c>
+      <c r="I96" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>49</v>
+      </c>
+      <c r="B97">
+        <v>0.38900000000000001</v>
+      </c>
+      <c r="C97" t="s">
+        <v>41</v>
+      </c>
+      <c r="F97" t="s">
+        <v>46</v>
+      </c>
+      <c r="G97">
+        <f>B99</f>
+        <v>2E-3</v>
+      </c>
+      <c r="H97">
+        <f>G97*6.1</f>
+        <v>1.2199999999999999E-2</v>
+      </c>
+      <c r="I97" t="s">
+        <v>76</v>
+      </c>
+      <c r="K97" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A98" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C98" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F98" t="s">
+        <v>10</v>
+      </c>
+      <c r="G98">
+        <v>2.4E-2</v>
+      </c>
+      <c r="H98">
+        <f>G98*6.1</f>
+        <v>0.1464</v>
+      </c>
+      <c r="I98" t="s">
+        <v>42</v>
+      </c>
+      <c r="K98" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L98" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="M98" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="N98" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>55</v>
+      </c>
+      <c r="B99">
+        <v>2E-3</v>
+      </c>
+      <c r="C99">
+        <f>B99*6.1</f>
+        <v>1.2199999999999999E-2</v>
+      </c>
+      <c r="D99" t="s">
+        <v>56</v>
+      </c>
+      <c r="K99" t="s">
+        <v>6</v>
+      </c>
+      <c r="L99" s="6">
+        <v>4.3999999999999997E-2</v>
+      </c>
+      <c r="M99">
+        <f>L99*6.1</f>
+        <v>0.26839999999999997</v>
+      </c>
+      <c r="N99" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>84</v>
+      </c>
+      <c r="B100">
+        <v>10.065</v>
+      </c>
+      <c r="C100">
+        <f>B100*6.1</f>
+        <v>61.396499999999996</v>
+      </c>
+      <c r="D100" t="s">
+        <v>85</v>
+      </c>
+      <c r="F100" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G100" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H100" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="I100" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="K100" t="s">
+        <v>70</v>
+      </c>
+      <c r="L100">
+        <f>G122</f>
+        <v>5.0830750541648664E-2</v>
+      </c>
+      <c r="M100">
+        <f>H122</f>
+        <v>0.26422990218203846</v>
+      </c>
+      <c r="N100" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F101" t="s">
+        <v>11</v>
+      </c>
+      <c r="G101">
+        <v>6.8000000000000005E-2</v>
+      </c>
+      <c r="H101">
+        <f>G101*2.49</f>
+        <v>0.16932000000000003</v>
+      </c>
+      <c r="I101" t="s">
+        <v>121</v>
+      </c>
+      <c r="K101" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L101" s="1">
+        <f>SUM(L99:L100)</f>
+        <v>9.4830750541648662E-2</v>
+      </c>
+      <c r="M101" s="1">
+        <f>SUM(M99:M100)</f>
+        <v>0.53262990218203843</v>
+      </c>
+      <c r="N101" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A102" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>5</v>
+      </c>
+      <c r="B103">
+        <v>1</v>
+      </c>
+      <c r="C103" t="s">
+        <v>79</v>
+      </c>
+      <c r="F103" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="L103">
+        <v>4.3999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B104" s="6">
+        <f>G132</f>
+        <v>7.0560000000000002E-5</v>
+      </c>
+      <c r="C104" t="s">
+        <v>80</v>
+      </c>
+      <c r="F104" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G104" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H104" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+      <c r="G105" s="6">
+        <f>G129</f>
+        <v>14.666666666666666</v>
+      </c>
+      <c r="H105" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A106" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F106" t="s">
+        <v>8</v>
+      </c>
+      <c r="G106" s="6">
+        <f>G105/40</f>
+        <v>0.36666666666666664</v>
+      </c>
+      <c r="H106" t="s">
+        <v>72</v>
+      </c>
+      <c r="K106" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A107" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C107" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D107" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F107" t="s">
+        <v>15</v>
+      </c>
+      <c r="G107">
+        <v>413.03911620000002</v>
+      </c>
+      <c r="H107" t="s">
+        <v>40</v>
+      </c>
+      <c r="K107" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L107" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="M107" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="N107" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>81</v>
+      </c>
+      <c r="B108">
+        <f>B93</f>
+        <v>1E-3</v>
+      </c>
+      <c r="C108">
+        <f>C93</f>
+        <v>6.0999999999999995E-3</v>
+      </c>
+      <c r="D108" t="s">
+        <v>75</v>
+      </c>
+      <c r="F108" t="s">
+        <v>13</v>
+      </c>
+      <c r="G108">
+        <v>4.5207999999999999E-4</v>
+      </c>
+      <c r="H108" t="s">
+        <v>73</v>
+      </c>
+      <c r="K108" t="s">
+        <v>7</v>
+      </c>
+      <c r="L108">
+        <f>L101*12/44*1000</f>
+        <v>25.862931965904178</v>
+      </c>
+      <c r="M108">
+        <f>M101*12/44*1000</f>
+        <v>145.26270059510139</v>
+      </c>
+      <c r="N108" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>82</v>
+      </c>
+      <c r="B109">
+        <f>B$55*B100</f>
+        <v>7.1018639999999994E-4</v>
+      </c>
+      <c r="C109">
+        <f>B$55*C100</f>
+        <v>4.3321370399999996E-3</v>
+      </c>
+      <c r="D109" t="s">
+        <v>75</v>
+      </c>
+      <c r="F109" t="s">
+        <v>98</v>
+      </c>
+      <c r="G109" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A110" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B110" s="1">
+        <f>SUM(B108:B109)</f>
+        <v>1.7101864E-3</v>
+      </c>
+      <c r="C110" s="1">
+        <f>SUM(C108:C109)</f>
+        <v>1.0432137039999999E-2</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F111" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="K111" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="L111" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="M111" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="E112" s="2"/>
+      <c r="F112" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G112" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="H112" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I112" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="K112" t="s">
+        <v>93</v>
+      </c>
+      <c r="L112">
+        <f>C93*G105</f>
+        <v>8.9466666666666653E-2</v>
+      </c>
+    </row>
+    <row r="113" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F113" t="s">
+        <v>63</v>
+      </c>
+      <c r="G113">
+        <f>G91/G105</f>
+        <v>1.315909090909091E-2</v>
+      </c>
+      <c r="H113">
+        <f>L$91*L$92</f>
+        <v>7.4853300000000001E-3</v>
+      </c>
+      <c r="I113">
+        <f>G113-H113</f>
+        <v>5.6737609090909101E-3</v>
+      </c>
+      <c r="K113" t="s">
+        <v>94</v>
+      </c>
+      <c r="L113">
+        <f>C109*G105</f>
+        <v>6.3538009919999985E-2</v>
+      </c>
+    </row>
+    <row r="114" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F114" t="s">
+        <v>67</v>
+      </c>
+      <c r="G114">
+        <f>G93/G106</f>
+        <v>1.0554545454545456</v>
+      </c>
+      <c r="H114">
+        <f t="shared" ref="H114:H115" si="2">L$91*L$92</f>
+        <v>7.4853300000000001E-3</v>
+      </c>
+      <c r="I114">
+        <f t="shared" ref="I114:I115" si="3">G114-H114</f>
+        <v>1.0479692154545457</v>
+      </c>
+      <c r="K114" t="s">
+        <v>95</v>
+      </c>
+      <c r="L114">
+        <f>H98*G106</f>
+        <v>5.3679999999999999E-2</v>
+      </c>
+    </row>
+    <row r="115" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F115" t="s">
+        <v>68</v>
+      </c>
+      <c r="G115">
+        <f>G92/G108</f>
+        <v>18076.446646611221</v>
+      </c>
+      <c r="H115">
+        <f t="shared" si="2"/>
+        <v>7.4853300000000001E-3</v>
+      </c>
+      <c r="I115">
+        <f t="shared" si="3"/>
+        <v>18076.439161281221</v>
+      </c>
+      <c r="K115" t="s">
+        <v>96</v>
+      </c>
+      <c r="L115">
+        <f>H101*G107*G108</f>
+        <v>3.1616568848705173E-2</v>
+      </c>
+    </row>
+    <row r="116" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="K116" t="s">
+        <v>97</v>
+      </c>
+      <c r="L116">
+        <f>M99</f>
+        <v>0.26839999999999997</v>
+      </c>
+    </row>
+    <row r="117" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F117" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="118" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F118" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G118" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="H118" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="I118" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="119" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F119" t="s">
+        <v>12</v>
+      </c>
+      <c r="G119">
+        <f>$G105*G97</f>
+        <v>2.9333333333333333E-2</v>
+      </c>
+      <c r="H119">
+        <f>$G105*H97</f>
+        <v>0.17893333333333331</v>
+      </c>
+      <c r="I119" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="120" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F120" t="s">
+        <v>14</v>
+      </c>
+      <c r="G120">
+        <f>$G107*G101*$G108</f>
+        <v>1.2697417208315329E-2</v>
+      </c>
+      <c r="H120">
+        <f>$G107*H101*$G108</f>
+        <v>3.1616568848705173E-2</v>
+      </c>
+      <c r="I120" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="121" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F121" t="s">
+        <v>74</v>
+      </c>
+      <c r="G121">
+        <f>$G98*G106</f>
+        <v>8.7999999999999988E-3</v>
+      </c>
+      <c r="H121">
+        <f>$H98*G106</f>
+        <v>5.3679999999999999E-2</v>
+      </c>
+      <c r="I121" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="122" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F122" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G122" s="1">
+        <f>SUM(G119:G121)</f>
+        <v>5.0830750541648664E-2</v>
+      </c>
+      <c r="H122" s="1">
+        <f>SUM(H119:H121)</f>
+        <v>0.26422990218203846</v>
+      </c>
+      <c r="I122" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="124" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F124" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="125" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F125" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G125" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H125" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="I125" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="126" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F126" t="s">
+        <v>102</v>
+      </c>
+      <c r="G126" t="e">
+        <f>G67/G68</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H126" t="s">
+        <v>105</v>
+      </c>
+      <c r="I126" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="127" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F127" t="s">
+        <v>109</v>
+      </c>
+      <c r="G127">
+        <v>40</v>
+      </c>
+      <c r="H127" t="s">
+        <v>105</v>
+      </c>
+      <c r="I127" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="128" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F128" t="s">
+        <v>110</v>
+      </c>
+      <c r="G128">
+        <f>G67</f>
+        <v>0</v>
+      </c>
+      <c r="H128" t="s">
+        <v>111</v>
+      </c>
+      <c r="I128" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="129" spans="6:10" x14ac:dyDescent="0.25">
+      <c r="F129" t="s">
+        <v>120</v>
+      </c>
+      <c r="G129">
+        <f>4*44/12</f>
+        <v>14.666666666666666</v>
+      </c>
+      <c r="H129" t="s">
+        <v>111</v>
+      </c>
+      <c r="I129" t="s">
+        <v>108</v>
+      </c>
+      <c r="J129" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="130" spans="6:10" x14ac:dyDescent="0.25">
+      <c r="F130" t="s">
+        <v>113</v>
+      </c>
+      <c r="G130">
+        <v>18</v>
+      </c>
+      <c r="H130" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="131" spans="6:10" x14ac:dyDescent="0.25">
+      <c r="F131" t="s">
+        <v>114</v>
+      </c>
+      <c r="G131">
+        <v>1.6</v>
+      </c>
+      <c r="H131" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="132" spans="6:10" x14ac:dyDescent="0.25">
+      <c r="F132" t="s">
+        <v>119</v>
+      </c>
+      <c r="G132">
+        <f>(G130+G131)*0.0036/1000</f>
+        <v>7.0560000000000002E-5</v>
+      </c>
+      <c r="H132" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="133" spans="6:10" x14ac:dyDescent="0.25">
+      <c r="F133" t="s">
+        <v>116</v>
+      </c>
+      <c r="G133">
+        <f>B66</f>
+        <v>0</v>
+      </c>
+      <c r="H133">
+        <f>C66</f>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K8">
-    <cfRule type="colorScale" priority="3">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4463,6 +6285,18 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K46">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K95">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
update elec supply data
</commit_message>
<xml_diff>
--- a/data/data_analysis/understanding TEW markets.xlsx
+++ b/data/data_analysis/understanding TEW markets.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\data\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7601D9F5-C6EC-4AEA-AFA7-70CD0754EB8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A1A2357-4FCD-4094-94FC-F387C2205271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{8111BAC2-3C26-4A41-BBD5-6F57C9F53EF0}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="125">
   <si>
     <t>2025 dollars</t>
   </si>
@@ -412,13 +412,16 @@
   </si>
   <si>
     <t>Updated Version</t>
+  </si>
+  <si>
+    <t>Electricity as %</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -470,6 +473,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -498,12 +508,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -514,11 +525,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4420,6 +4433,13 @@
       <c r="I30" s="5" t="s">
         <v>2</v>
       </c>
+      <c r="K30" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="L30" s="8">
+        <f>L26/SUM(L25:L29)</f>
+        <v>0.65334941489381693</v>
+      </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F31" t="s">
@@ -5186,6 +5206,13 @@
     <row r="68" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F68" s="4" t="s">
         <v>69</v>
+      </c>
+      <c r="K68" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="L68" s="8">
+        <f>L64/SUM(L63:L67)</f>
+        <v>0.13502614278792191</v>
       </c>
     </row>
     <row r="69" spans="6:12" x14ac:dyDescent="0.25">
@@ -6309,7 +6336,8 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>